<commit_message>
BuilderRenamer updates Renamer can now rename Seal Models Renamer now renamed class names in all models Fixed misspelled Quicksilver seal class name
</commit_message>
<xml_diff>
--- a/demon_pie.xlsx
+++ b/demon_pie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4b5af9c88eeda555/Documents/GitHub/demon-flip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="333" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6E7F27B2-EC7F-4B24-8B36-9938502C3A4D}"/>
+  <xr:revisionPtr revIDLastSave="390" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B532F5B6-2B9E-46F9-BCC5-A4532797E831}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{98FBD9DA-F62C-4058-B636-95D985AB8E5E}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="213" uniqueCount="43">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="47">
   <si>
     <t>Gluttony</t>
   </si>
@@ -169,6 +168,18 @@
   </si>
   <si>
     <t>Self Damage</t>
+  </si>
+  <si>
+    <t>Spin Advantage</t>
+  </si>
+  <si>
+    <t>Stall</t>
+  </si>
+  <si>
+    <t>Copy</t>
+  </si>
+  <si>
+    <t>Removal</t>
   </si>
 </sst>
 </file>
@@ -313,7 +324,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -332,6 +343,8 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1085,36 +1098,50 @@
       </c>
     </row>
     <row r="21" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="B21" t="s">
-        <v>40</v>
-      </c>
-      <c r="C21" t="s">
-        <v>35</v>
-      </c>
-      <c r="D21" s="17" t="s">
-        <v>36</v>
-      </c>
-      <c r="E21" t="s">
-        <v>34</v>
-      </c>
-      <c r="F21" t="s">
-        <v>37</v>
-      </c>
-      <c r="G21" t="s">
-        <v>39</v>
-      </c>
-      <c r="H21" t="s">
-        <v>38</v>
-      </c>
       <c r="I21" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B22" t="s">
+        <v>40</v>
+      </c>
+      <c r="C22" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E22" t="s">
+        <v>34</v>
+      </c>
       <c r="F22" t="s">
+        <v>37</v>
+      </c>
+      <c r="G22" t="s">
+        <v>39</v>
+      </c>
+      <c r="H22" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="B23" t="s">
+        <v>46</v>
+      </c>
+      <c r="C23" t="s">
+        <v>45</v>
+      </c>
+      <c r="D23" t="s">
+        <v>44</v>
+      </c>
+      <c r="E23" t="s">
+        <v>43</v>
+      </c>
+      <c r="F23" t="s">
         <v>42</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H23" t="s">
         <v>41</v>
       </c>
     </row>
@@ -1145,243 +1172,228 @@
       <c r="A29" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="B29" t="s">
-        <v>4</v>
-      </c>
-      <c r="C29" t="s">
-        <v>1</v>
-      </c>
-      <c r="D29" t="s">
-        <v>5</v>
-      </c>
-      <c r="E29" t="s">
-        <v>6</v>
-      </c>
-      <c r="F29" t="s">
-        <v>0</v>
-      </c>
-      <c r="G29" t="s">
-        <v>3</v>
-      </c>
-      <c r="H29" t="s">
-        <v>2</v>
+      <c r="B29" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="E29" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H29" s="12" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="B30" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C30" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F30" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="G30" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="H30" s="3" t="s">
-        <v>12</v>
+      <c r="B30" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C30" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>20</v>
       </c>
     </row>
     <row r="31" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A31" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D31" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="E31" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F31" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G31" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="H31" s="5" t="s">
-        <v>14</v>
+      <c r="B31" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="C31" s="11" t="s">
+        <v>22</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E31" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="G31" s="14" t="s">
+        <v>25</v>
+      </c>
+      <c r="H31" s="9" t="s">
+        <v>18</v>
       </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" s="13" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="D32" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="E32" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="F32" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="H32" s="6" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33" s="11" t="s">
         <v>22</v>
       </c>
+      <c r="B33" t="s">
+        <v>40</v>
+      </c>
+      <c r="C33" t="s">
+        <v>35</v>
+      </c>
+      <c r="D33" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="E33" t="s">
+        <v>34</v>
+      </c>
+      <c r="F33" t="s">
+        <v>37</v>
+      </c>
+      <c r="G33" t="s">
+        <v>39</v>
+      </c>
+      <c r="H33" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="B34" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="C34" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="E34" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="G34" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H34" s="13" t="s">
-        <v>20</v>
+      <c r="B34" t="s">
+        <v>34</v>
+      </c>
+      <c r="C34" t="s">
+        <v>37</v>
+      </c>
+      <c r="D34" t="s">
+        <v>38</v>
+      </c>
+      <c r="E34" t="s">
+        <v>35</v>
+      </c>
+      <c r="F34" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" t="s">
+        <v>39</v>
+      </c>
+      <c r="H34" s="17" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B35" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="F35" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G35" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>24</v>
+      <c r="B35" s="17" t="s">
+        <v>36</v>
+      </c>
+      <c r="C35" t="s">
+        <v>40</v>
+      </c>
+      <c r="D35" t="s">
+        <v>37</v>
+      </c>
+      <c r="E35" t="s">
+        <v>38</v>
+      </c>
+      <c r="F35" t="s">
+        <v>34</v>
+      </c>
+      <c r="G35" t="s">
+        <v>39</v>
+      </c>
+      <c r="H35" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B36" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="G36" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="H36" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="B36" s="18"/>
+      <c r="C36" s="18"/>
+      <c r="D36" s="18"/>
+      <c r="E36" s="18"/>
+      <c r="F36" s="18"/>
+      <c r="G36" s="18"/>
+      <c r="H36" s="19"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="G37" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="B37" s="18"/>
+      <c r="C37" s="18"/>
+      <c r="D37" s="18"/>
+      <c r="E37" s="18"/>
+      <c r="F37" s="18"/>
+      <c r="G37" s="18"/>
+      <c r="H37" s="18"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>21</v>
       </c>
+      <c r="B38" s="18"/>
+      <c r="C38" s="18"/>
+      <c r="D38" s="18"/>
+      <c r="E38" s="18"/>
+      <c r="F38" s="18"/>
+      <c r="G38" s="18"/>
+      <c r="H38" s="18"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C39" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D39" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="E39" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" s="13" t="s">
-        <v>20</v>
-      </c>
+      <c r="B39" s="18"/>
+      <c r="C39" s="18"/>
+      <c r="D39" s="19"/>
+      <c r="E39" s="18"/>
+      <c r="F39" s="18"/>
+      <c r="G39" s="18"/>
+      <c r="H39" s="18"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="D40" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E40" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="F40" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="G40" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H40" s="12" t="s">
-        <v>24</v>
-      </c>
+      <c r="B40" s="18"/>
+      <c r="C40" s="18"/>
+      <c r="D40" s="18"/>
+      <c r="E40" s="18"/>
+      <c r="F40" s="19"/>
+      <c r="G40" s="18"/>
+      <c r="H40" s="18"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D41" s="8" t="s">
-        <v>17</v>
-      </c>
-      <c r="E41" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="F41" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H41" s="11" t="s">
-        <v>22</v>
-      </c>
+      <c r="B41" s="18"/>
+      <c r="C41" s="18"/>
+      <c r="D41" s="18"/>
+      <c r="E41" s="18"/>
+      <c r="F41" s="18"/>
+      <c r="G41" s="18"/>
+      <c r="H41" s="19"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added 2 New Abilities for Sloth Added 2 New Rings for Sloth Added 2 New Seals Added amoutPointer to onAfterSpinChanged trigger Changed MatchState.spin_changed to a CFSignal and added delay after spin change in AdvantageBar Added PopperNodes to player spin labels in AdvantageBar Updated Lives Texture Reduced wait time after a seal is broken Nerfed FogOfMind to no longer stamp AquaFortis Fixed player being able to activate an ability before actionable Fixed ring nodes being on the same z-index as finger sprites Added flavor key to eng.json for Rings and Seals
</commit_message>
<xml_diff>
--- a/demon_pie.xlsx
+++ b/demon_pie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4b5af9c88eeda555/Documents/GitHub/demon-flip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="390" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B532F5B6-2B9E-46F9-BCC5-A4532797E831}"/>
+  <xr:revisionPtr revIDLastSave="434" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31AD88CE-9267-44CC-B2DB-F5C0FA632403}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{98FBD9DA-F62C-4058-B636-95D985AB8E5E}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="52">
   <si>
     <t>Gluttony</t>
   </si>
@@ -180,6 +181,21 @@
   </si>
   <si>
     <t>Removal</t>
+  </si>
+  <si>
+    <t>Sound</t>
+  </si>
+  <si>
+    <t>Smell</t>
+  </si>
+  <si>
+    <t>Touch</t>
+  </si>
+  <si>
+    <t>Sight</t>
+  </si>
+  <si>
+    <t>Taste</t>
   </si>
 </sst>
 </file>
@@ -324,7 +340,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -343,8 +359,7 @@
     <xf numFmtId="0" fontId="0" fillId="16" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -752,6 +767,21 @@
       <c r="H2" s="5" t="s">
         <v>14</v>
       </c>
+      <c r="J2" t="s">
+        <v>47</v>
+      </c>
+      <c r="K2" t="s">
+        <v>48</v>
+      </c>
+      <c r="L2" t="s">
+        <v>49</v>
+      </c>
+      <c r="M2" t="s">
+        <v>50</v>
+      </c>
+      <c r="N2" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -804,6 +834,29 @@
       <c r="H4" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="J4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="K4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="M4" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="N4" s="6" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="L5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B6" s="6" t="s">
@@ -827,6 +880,15 @@
       <c r="H6" s="5" t="s">
         <v>14</v>
       </c>
+      <c r="J6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="K6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="N6" s="3" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B7" s="1" t="s">
@@ -850,6 +912,12 @@
       <c r="H7" s="4" t="s">
         <v>13</v>
       </c>
+      <c r="L7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M7" s="1" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
@@ -873,10 +941,34 @@
       <c r="H8" s="3" t="s">
         <v>12</v>
       </c>
+      <c r="J8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="L8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="M8" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>10</v>
+      </c>
+      <c r="J9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="K9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="L9" s="5" t="s">
+        <v>14</v>
       </c>
     </row>
     <row r="10" spans="1:14" x14ac:dyDescent="0.25">
@@ -1333,67 +1425,29 @@
       <c r="A36" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="19"/>
+      <c r="H36" s="18"/>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
         <v>26</v>
       </c>
-      <c r="B37" s="18"/>
-      <c r="C37" s="18"/>
-      <c r="D37" s="18"/>
-      <c r="E37" s="18"/>
-      <c r="F37" s="18"/>
-      <c r="G37" s="18"/>
-      <c r="H37" s="18"/>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>21</v>
       </c>
-      <c r="B38" s="18"/>
-      <c r="C38" s="18"/>
-      <c r="D38" s="18"/>
-      <c r="E38" s="18"/>
-      <c r="F38" s="18"/>
-      <c r="G38" s="18"/>
-      <c r="H38" s="18"/>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="19"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
+      <c r="D39" s="18"/>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B40" s="18"/>
-      <c r="C40" s="18"/>
-      <c r="D40" s="18"/>
-      <c r="E40" s="18"/>
-      <c r="F40" s="19"/>
-      <c r="G40" s="18"/>
-      <c r="H40" s="18"/>
+      <c r="F40" s="18"/>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="B41" s="18"/>
-      <c r="C41" s="18"/>
-      <c r="D41" s="18"/>
-      <c r="E41" s="18"/>
-      <c r="F41" s="18"/>
-      <c r="G41" s="18"/>
-      <c r="H41" s="19"/>
+      <c r="H41" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Updated art to match Demon colors
</commit_message>
<xml_diff>
--- a/demon_pie.xlsx
+++ b/demon_pie.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4b5af9c88eeda555/Documents/GitHub/demon-flip/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="434" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{31AD88CE-9267-44CC-B2DB-F5C0FA632403}"/>
+  <xr:revisionPtr revIDLastSave="468" documentId="8_{72EAA511-0279-44C2-87F7-2AD018803773}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25807E55-E1A6-4B73-9B33-CE1DE252B18E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{98FBD9DA-F62C-4058-B636-95D985AB8E5E}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -40,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="223" uniqueCount="53">
   <si>
     <t>Gluttony</t>
   </si>
@@ -196,6 +195,9 @@
   </si>
   <si>
     <t>Taste</t>
+  </si>
+  <si>
+    <t>Darkness</t>
   </si>
 </sst>
 </file>
@@ -340,7 +342,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
@@ -360,6 +362,7 @@
     <xf numFmtId="0" fontId="0" fillId="17" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1196,25 +1199,25 @@
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
       <c r="B22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" t="s">
         <v>35</v>
       </c>
       <c r="D22" s="17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E22" t="s">
+        <v>37</v>
+      </c>
+      <c r="F22" t="s">
+        <v>40</v>
+      </c>
+      <c r="G22" t="s">
+        <v>34</v>
+      </c>
+      <c r="H22" t="s">
         <v>36</v>
-      </c>
-      <c r="E22" t="s">
-        <v>34</v>
-      </c>
-      <c r="F22" t="s">
-        <v>37</v>
-      </c>
-      <c r="G22" t="s">
-        <v>39</v>
-      </c>
-      <c r="H22" t="s">
-        <v>38</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1348,25 +1351,25 @@
         <v>22</v>
       </c>
       <c r="B33" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="C33" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="D33" s="17" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="E33" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="F33" t="s">
-        <v>37</v>
-      </c>
-      <c r="G33" t="s">
-        <v>39</v>
-      </c>
-      <c r="H33" t="s">
-        <v>38</v>
+        <v>52</v>
+      </c>
+      <c r="G33" s="19" t="s">
+        <v>25</v>
+      </c>
+      <c r="H33" s="19" t="s">
+        <v>24</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -1374,25 +1377,25 @@
         <v>24</v>
       </c>
       <c r="B34" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="C34" t="s">
-        <v>37</v>
-      </c>
-      <c r="D34" t="s">
-        <v>38</v>
+        <v>52</v>
+      </c>
+      <c r="D34" s="19" t="s">
+        <v>24</v>
       </c>
       <c r="E34" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
       <c r="F34" t="s">
-        <v>40</v>
-      </c>
-      <c r="G34" t="s">
-        <v>39</v>
+        <v>22</v>
+      </c>
+      <c r="G34" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="H34" s="17" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -1400,25 +1403,25 @@
         <v>23</v>
       </c>
       <c r="B35" s="17" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="C35" t="s">
-        <v>40</v>
+        <v>22</v>
       </c>
       <c r="D35" t="s">
-        <v>37</v>
-      </c>
-      <c r="E35" t="s">
-        <v>38</v>
+        <v>52</v>
+      </c>
+      <c r="E35" s="19" t="s">
+        <v>24</v>
       </c>
       <c r="F35" t="s">
-        <v>34</v>
-      </c>
-      <c r="G35" t="s">
-        <v>39</v>
+        <v>17</v>
+      </c>
+      <c r="G35" s="19" t="s">
+        <v>25</v>
       </c>
       <c r="H35" t="s">
-        <v>35</v>
+        <v>18</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>